<commit_message>
update 2nd testchip plan
</commit_message>
<xml_diff>
--- a/Template/KWS9_SOW.xlsx
+++ b/Template/KWS9_SOW.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSYS2\home\yiqis\github\MD_Group\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BD86DA-3940-4123-9D39-96DE102D8572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DC0B26-0C7A-4A43-9D1C-F26E6B7EE46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 2" sheetId="4" r:id="rId1"/>
@@ -25,6 +25,9 @@
     <sheet name="Table 7" sheetId="15" r:id="rId10"/>
     <sheet name="Table 8" sheetId="16" r:id="rId11"/>
     <sheet name="Table 9" sheetId="17" r:id="rId12"/>
+    <sheet name="Table 10" sheetId="19" r:id="rId13"/>
+    <sheet name="Table 11" sheetId="20" r:id="rId14"/>
+    <sheet name="Table 12" sheetId="21" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="177">
   <si>
     <t>Table Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -390,10 +393,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Table: 封装测试计划</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Testchip Package</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -431,10 +430,6 @@
   </si>
   <si>
     <t>T0 + 3.5 month</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Table: 测试片开发计划</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -455,8 +450,146 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>PDK Version</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Metal Stack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TFBGA(TBD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>16k</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>32k</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>64k</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.110</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.124</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.185</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.274</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8T2P</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KWS9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GF22nm(TBD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~5mm*5mm(TBD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/10/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/8/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/8/22</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D1240 HC6T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D1850 8T2P</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nominal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FuncCmax</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TT0P65V0P8V25CTT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TT0P65V0P8V85CTT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1P8M(TBD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/11/25</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/11/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/8/25</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/10/10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/11/30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Table: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第一阶段</t>
     </r>
     <r>
       <rPr>
@@ -470,131 +603,112 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PDK Version</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Metal Stack</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TFBGA(TBD)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>16k</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>32k</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>64k</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.110</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.124</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.185</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.274</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>8T2P</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>KWS9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>GF22nm(TBD)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>~5mm*5mm(TBD)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/10/15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/8/15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/8/22</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>D1240 HC6T</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>D1850 8T2P</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>P3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>P4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Nominal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FuncCmax</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TT0P65V0P8V25CTT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TT0P65V0P8V85CTT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1P8M(TBD)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/11/25</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/11/15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/8/25</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/10/10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026/11/30</t>
+    <t>Table: 第一阶段测试片开发计划</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table: 第一阶段封装测试计划</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Table: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>第二阶段</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>测试片信息</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KWS11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table: 第二阶段测试片开发计划</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table: 第二阶段封装测试计划</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/12/01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/12/05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/3/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/3/20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/12/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/1/31</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/1/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/2/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/12/20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026/12/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/3/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/6/25</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/6/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/6/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2027/6/30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOI 22nm(TBD)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -602,7 +716,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -668,6 +782,13 @@
       <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="1"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1219,16 +1340,16 @@
         <v>17</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1236,19 +1357,19 @@
         <v>33</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C2" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>131</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1275,27 +1396,27 @@
         <v>89</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A3" s="22"/>
       <c r="B3" s="15" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
@@ -1304,7 +1425,7 @@
         <v>90</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
@@ -1313,7 +1434,7 @@
         <v>91</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1355,7 +1476,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>119</v>
+        <v>155</v>
       </c>
       <c r="B2" s="10">
         <v>1</v>
@@ -1397,7 +1518,7 @@
         <v>107</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1409,10 +1530,10 @@
         <v>95</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -1424,10 +1545,10 @@
         <v>96</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1439,10 +1560,10 @@
         <v>97</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1454,10 +1575,10 @@
         <v>98</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1469,10 +1590,10 @@
         <v>99</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -1484,10 +1605,10 @@
         <v>100</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1520,21 +1641,21 @@
         <v>101</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="B2" s="10">
         <v>1</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1543,10 +1664,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1555,10 +1676,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>116</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1567,10 +1688,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1579,10 +1700,347 @@
         <v>5</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A6"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E2A6B2C-A44A-4428-A072-3E207A8A5358}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.125" customWidth="1"/>
+    <col min="2" max="2" width="14.25" customWidth="1"/>
+    <col min="3" max="3" width="20.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="22"/>
+      <c r="B3" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="22"/>
+      <c r="B4" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="23"/>
+      <c r="B5" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A5"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93CFDE81-AA5C-4CAA-9A39-B64FFD0E7B6C}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.25" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="13.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="B2" s="10">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="16"/>
+      <c r="B3" s="10">
+        <v>2</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="16"/>
+      <c r="B4" s="10">
+        <v>3</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="16"/>
+      <c r="B5" s="10">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="16"/>
+      <c r="B6" s="10">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="16"/>
+      <c r="B7" s="10">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="10">
+        <v>7</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="16"/>
+      <c r="B9" s="10">
+        <v>8</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="16"/>
+      <c r="B10" s="10">
+        <v>9</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A10"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0461EA20-6944-4893-8643-E20B1C2A3F0E}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.25" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="13.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" s="10">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>111</v>
       </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="16"/>
+      <c r="B3" s="10">
+        <v>2</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="16"/>
+      <c r="B4" s="10">
+        <v>3</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="16"/>
+      <c r="B5" s="10">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="16"/>
+      <c r="B6" s="10">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>110</v>
+      </c>
       <c r="D6" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1620,7 +2078,7 @@
     </row>
     <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>15</v>
@@ -1629,7 +2087,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1641,31 +2099,31 @@
         <v>18</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="16"/>
       <c r="B4" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="16"/>
       <c r="B5" s="10" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1712,7 +2170,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1724,31 +2182,31 @@
         <v>18</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18"/>
       <c r="B4" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
       <c r="B5" s="10" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2174,7 +2632,7 @@
         <v>256</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -2204,7 +2662,7 @@
         <v>256</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -2234,7 +2692,7 @@
         <v>256</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -2294,7 +2752,7 @@
         <v>128</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -2324,7 +2782,7 @@
         <v>128</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -2354,7 +2812,7 @@
         <v>128</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -2862,7 +3320,7 @@
         <v>25</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -2883,7 +3341,7 @@
         <v>85</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -2904,7 +3362,7 @@
         <v>-40</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -2925,7 +3383,7 @@
         <v>125</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -2946,7 +3404,7 @@
         <v>-40</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -2967,13 +3425,13 @@
         <v>125</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="16"/>
       <c r="B8" s="10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>40</v>
@@ -2988,13 +3446,13 @@
         <v>25</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="16"/>
       <c r="B9" s="10" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>40</v>
@@ -3009,7 +3467,7 @@
         <v>85</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>